<commit_message>
Login and add user completed search pending git add .
</commit_message>
<xml_diff>
--- a/src/main/resources/testData/qdPM_dataSheet.xlsx
+++ b/src/main/resources/testData/qdPM_dataSheet.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="22188" windowHeight="9000" activeTab="1"/>
+    <workbookView windowWidth="14375" windowHeight="9455" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Admin_TC" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="40">
   <si>
     <t>CRUD opertations for client user using Admin user</t>
   </si>
@@ -102,13 +102,13 @@
     <t>Field</t>
   </si>
   <si>
-    <t>Data</t>
+    <t>Values</t>
   </si>
   <si>
     <t>Active</t>
   </si>
   <si>
-    <t>yes</t>
+    <t>No</t>
   </si>
   <si>
     <t>Group</t>
@@ -142,6 +142,12 @@
   </si>
   <si>
     <t>Hindi</t>
+  </si>
+  <si>
+    <t>Notify</t>
+  </si>
+  <si>
+    <t>Yes</t>
   </si>
 </sst>
 </file>
@@ -779,14 +785,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="6" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1330,166 +1336,166 @@
   </cols>
   <sheetData>
     <row r="1" ht="28.8" spans="1:3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="4"/>
+      <c r="C2" s="2"/>
     </row>
     <row r="3" spans="1:3">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="4"/>
+      <c r="C3" s="2"/>
     </row>
     <row r="4" ht="28.8" spans="1:3">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="3"/>
+      <c r="C4" s="4"/>
     </row>
     <row r="5" spans="1:3">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="3"/>
+      <c r="C5" s="4"/>
     </row>
     <row r="6" ht="28.8" spans="1:3">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="7" ht="28.8" spans="1:3">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="3"/>
+      <c r="C7" s="4"/>
     </row>
     <row r="8" spans="1:3">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="4"/>
+      <c r="C8" s="2"/>
     </row>
     <row r="9" ht="28.8" spans="1:3">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="4"/>
+      <c r="C9" s="2"/>
     </row>
     <row r="10" ht="28.8" spans="1:3">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="4"/>
+      <c r="C10" s="2"/>
     </row>
     <row r="11" ht="28.8" spans="1:3">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="4"/>
+      <c r="C11" s="2"/>
     </row>
     <row r="12" ht="43.2" spans="1:3">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C12" s="4"/>
+      <c r="C12" s="2"/>
     </row>
     <row r="13" ht="28.8" spans="1:3">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="4"/>
+      <c r="C13" s="2"/>
     </row>
     <row r="14" ht="28.8" spans="1:3">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C14" s="4"/>
+      <c r="C14" s="2"/>
     </row>
     <row r="15" spans="1:3">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C15" s="4"/>
+      <c r="C15" s="2"/>
     </row>
     <row r="16" spans="1:3">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="4"/>
+      <c r="C16" s="2"/>
     </row>
     <row r="17" ht="28.8" spans="1:3">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="4"/>
+      <c r="C17" s="2"/>
     </row>
     <row r="18" ht="28.8" spans="1:3">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C18" s="4"/>
+      <c r="C18" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1500,9 +1506,10 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="7" outlineLevelCol="1"/>
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <cols>
+    <col min="1" max="1" width="20.2222222222222" customWidth="1"/>
     <col min="2" max="2" width="26.6666666666667" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1510,7 +1517,7 @@
       <c r="A1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>24</v>
       </c>
     </row>
@@ -1550,7 +1557,7 @@
       <c r="A6" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>34</v>
       </c>
     </row>
@@ -1568,6 +1575,14 @@
       </c>
       <c r="B8" s="1" t="s">
         <v>37</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Test cases written..working on update the data
</commit_message>
<xml_diff>
--- a/src/main/resources/testData/qdPM_dataSheet.xlsx
+++ b/src/main/resources/testData/qdPM_dataSheet.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="14375" windowHeight="9455" activeTab="1"/>
+    <workbookView windowWidth="22188" windowHeight="9000" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Admin_TC" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="42">
   <si>
     <t>CRUD opertations for client user using Admin user</t>
   </si>
@@ -148,6 +148,12 @@
   </si>
   <si>
     <t>Yes</t>
+  </si>
+  <si>
+    <t>Update Language</t>
+  </si>
+  <si>
+    <t>English</t>
   </si>
 </sst>
 </file>
@@ -778,7 +784,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -790,6 +796,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="6" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -1336,7 +1345,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28.8" spans="1:3">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
@@ -1346,7 +1355,7 @@
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="5" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="2"/>
@@ -1355,7 +1364,7 @@
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="5" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="2"/>
@@ -1364,28 +1373,28 @@
       <c r="A4" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="4"/>
+      <c r="C4" s="5"/>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="4"/>
+      <c r="C5" s="5"/>
     </row>
     <row r="6" ht="28.8" spans="1:3">
       <c r="A6" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="5" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1393,16 +1402,16 @@
       <c r="A7" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="4"/>
+      <c r="C7" s="5"/>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="5" t="s">
         <v>10</v>
       </c>
       <c r="C8" s="2"/>
@@ -1411,7 +1420,7 @@
       <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="5" t="s">
         <v>11</v>
       </c>
       <c r="C9" s="2"/>
@@ -1420,7 +1429,7 @@
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="5" t="s">
         <v>12</v>
       </c>
       <c r="C10" s="2"/>
@@ -1429,7 +1438,7 @@
       <c r="A11" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C11" s="2"/>
@@ -1438,7 +1447,7 @@
       <c r="A12" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C12" s="2"/>
@@ -1447,7 +1456,7 @@
       <c r="A13" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="5" t="s">
         <v>15</v>
       </c>
       <c r="C13" s="2"/>
@@ -1456,7 +1465,7 @@
       <c r="A14" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="5" t="s">
         <v>17</v>
       </c>
       <c r="C14" s="2"/>
@@ -1465,7 +1474,7 @@
       <c r="A15" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="5" t="s">
         <v>18</v>
       </c>
       <c r="C15" s="2"/>
@@ -1474,7 +1483,7 @@
       <c r="A16" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="5" t="s">
         <v>20</v>
       </c>
       <c r="C16" s="2"/>
@@ -1483,7 +1492,7 @@
       <c r="A17" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="5" t="s">
         <v>21</v>
       </c>
       <c r="C17" s="2"/>
@@ -1492,7 +1501,7 @@
       <c r="A18" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="5" t="s">
         <v>22</v>
       </c>
       <c r="C18" s="2"/>
@@ -1506,10 +1515,10 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="20.2222222222222" customWidth="1"/>
+    <col min="1" max="1" width="22.8888888888889" customWidth="1"/>
     <col min="2" max="2" width="26.6666666666667" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1583,6 +1592,14 @@
       </c>
       <c r="B9" s="2" t="s">
         <v>39</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
TC creation pending git add . picking up wrong name sumit instead of test user in update phone number test case
</commit_message>
<xml_diff>
--- a/src/main/resources/testData/qdPM_dataSheet.xlsx
+++ b/src/main/resources/testData/qdPM_dataSheet.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="49">
   <si>
     <t>CRUD opertations for client user using Admin user</t>
   </si>
@@ -39,16 +39,22 @@
     <t>Navigate to Login page</t>
   </si>
   <si>
+    <t>TC_1</t>
+  </si>
+  <si>
     <t>Login using admin credentials</t>
   </si>
   <si>
-    <t>Try to login with incorrect credentials</t>
+    <t>Get the User Name and validate the Admin user</t>
   </si>
   <si>
     <t>Navigate to add user page</t>
   </si>
   <si>
-    <t xml:space="preserve">Create a client user </t>
+    <t>TC_2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create a Developer user </t>
   </si>
   <si>
     <t>Pick data from excel sheet using data provider and apache POI</t>
@@ -60,9 +66,15 @@
     <t>Send login details to user email checkbox is checked</t>
   </si>
   <si>
+    <t xml:space="preserve">Pending </t>
+  </si>
+  <si>
     <t>Search user with user name</t>
   </si>
   <si>
+    <t>TC_3</t>
+  </si>
+  <si>
     <t>Validate user name from the data table</t>
   </si>
   <si>
@@ -84,6 +96,9 @@
     <t>Update some details of the client</t>
   </si>
   <si>
+    <t>TC_4</t>
+  </si>
+  <si>
     <t>Validate the updated details</t>
   </si>
   <si>
@@ -93,6 +108,9 @@
     <t>Delete the created client user</t>
   </si>
   <si>
+    <t>TC_5</t>
+  </si>
+  <si>
     <t>Verify on the data table if user exisist</t>
   </si>
   <si>
@@ -114,19 +132,19 @@
     <t>Group</t>
   </si>
   <si>
-    <t>Client</t>
+    <t>Developer</t>
   </si>
   <si>
     <t>Full Name</t>
   </si>
   <si>
-    <t>Client user</t>
+    <t>Test user</t>
   </si>
   <si>
     <t>Password</t>
   </si>
   <si>
-    <t>sumitc</t>
+    <t>sumitd</t>
   </si>
   <si>
     <t>Email</t>
@@ -138,6 +156,9 @@
     <t>Phone</t>
   </si>
   <si>
+    <t>9868988188</t>
+  </si>
+  <si>
     <t>Language</t>
   </si>
   <si>
@@ -150,10 +171,10 @@
     <t>Yes</t>
   </si>
   <si>
-    <t>Update Language</t>
-  </si>
-  <si>
-    <t>English</t>
+    <t>Updated Phone</t>
+  </si>
+  <si>
+    <t>9711678967</t>
   </si>
 </sst>
 </file>
@@ -784,7 +805,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -797,11 +818,14 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="6" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" quotePrefix="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1336,8 +1360,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C18"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="2"/>
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="3"/>
   <cols>
     <col min="1" max="1" width="28.7777777777778" customWidth="1"/>
     <col min="2" max="2" width="27.2222222222222" customWidth="1"/>
@@ -1345,164 +1369,209 @@
   </cols>
   <sheetData>
     <row r="1" ht="28.8" spans="1:3">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:4">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="4" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="2"/>
-    </row>
-    <row r="3" spans="1:3">
+      <c r="D2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="2"/>
+      <c r="D3" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="2"/>
-    </row>
-    <row r="4" ht="28.8" spans="1:3">
+    </row>
+    <row r="4" ht="28.8" spans="1:4">
       <c r="A4" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" s="5"/>
-    </row>
-    <row r="5" spans="1:3">
+      <c r="B4" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="4"/>
+      <c r="D4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
       <c r="A5" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" s="5"/>
-    </row>
-    <row r="6" ht="28.8" spans="1:3">
+      <c r="B5" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="4"/>
+      <c r="D5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" ht="28.8" spans="1:4">
       <c r="A6" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" s="5" t="s">
+      <c r="B6" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="7" ht="28.8" spans="1:3">
+    <row r="7" ht="28.8" spans="1:4">
       <c r="A7" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C7" s="5"/>
-    </row>
-    <row r="8" spans="1:3">
+        <v>10</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="4"/>
+      <c r="D7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
       <c r="A8" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8" s="5" t="s">
         <v>10</v>
       </c>
+      <c r="B8" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="C8" s="2"/>
-    </row>
-    <row r="9" ht="28.8" spans="1:3">
+      <c r="D8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" ht="28.8" spans="1:4">
       <c r="A9" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>15</v>
       </c>
       <c r="C9" s="2"/>
-    </row>
-    <row r="10" ht="28.8" spans="1:3">
+      <c r="D9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" ht="28.8" spans="1:4">
       <c r="A10" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B10" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="2"/>
+      <c r="D10" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="2"/>
-    </row>
-    <row r="11" ht="28.8" spans="1:3">
+    </row>
+    <row r="11" ht="28.8" spans="1:4">
       <c r="A11" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>13</v>
+        <v>10</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>17</v>
       </c>
       <c r="C11" s="2"/>
-    </row>
-    <row r="12" ht="43.2" spans="1:3">
+      <c r="D11" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" ht="43.2" spans="1:4">
       <c r="A12" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>14</v>
+        <v>10</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>18</v>
       </c>
       <c r="C12" s="2"/>
-    </row>
-    <row r="13" ht="28.8" spans="1:3">
+      <c r="D12" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" ht="28.8" spans="1:4">
       <c r="A13" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>15</v>
+        <v>10</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>19</v>
       </c>
       <c r="C13" s="2"/>
-    </row>
-    <row r="14" ht="28.8" spans="1:3">
+      <c r="D13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" ht="28.8" spans="1:4">
       <c r="A14" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>17</v>
+        <v>20</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>21</v>
       </c>
       <c r="C14" s="2"/>
-    </row>
-    <row r="15" spans="1:3">
+      <c r="D14" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
       <c r="A15" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>18</v>
+        <v>20</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>23</v>
       </c>
       <c r="C15" s="2"/>
-    </row>
-    <row r="16" spans="1:3">
+      <c r="D15" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
       <c r="A16" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>20</v>
+        <v>24</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="C16" s="2"/>
+      <c r="D16" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="17" ht="28.8" spans="1:3">
       <c r="A17" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>21</v>
+        <v>24</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>27</v>
       </c>
       <c r="C17" s="2"/>
     </row>
     <row r="18" ht="28.8" spans="1:3">
       <c r="A18" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>22</v>
+        <v>24</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>28</v>
       </c>
       <c r="C18" s="2"/>
     </row>
@@ -1524,82 +1593,82 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B7" s="1">
-        <v>98988888</v>
+        <v>41</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="2" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
     </row>
     <row r="10" spans="1:2">
-      <c r="A10" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>41</v>
+      <c r="A10" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>